<commit_message>
rerun the pipeline end to end so every report, workbook and figure matches the code
</commit_message>
<xml_diff>
--- a/01_Preprocess/02_Quantification/c_data/02_quantify.xlsx
+++ b/01_Preprocess/02_Quantification/c_data/02_quantify.xlsx
@@ -7,8 +7,9 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="dpc_parameters" sheetId="1" r:id="rId1"/>
-    <sheet name="protein_quality" sheetId="2" r:id="rId2"/>
+    <sheet name="overview" sheetId="1" r:id="rId1"/>
+    <sheet name="dpc_parameters" sheetId="2" r:id="rId2"/>
+    <sheet name="protein_quality" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -352,27 +353,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>intercept</t>
+          <t>sheet</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>slope</t>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>-8.958339019700954</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dpc_parameters</t>
+        </is>
       </c>
       <c r="B2">
-        <v>0.4883638963892026</v>
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Intercept and slope of the fitted detection probability curve</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>protein_quality</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>3042</v>
+      </c>
+      <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Per protein: precursors, observed proportion, mean abundance, standard error, observations</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -382,6 +421,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>intercept</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>slope</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>-8.958339019700954</v>
+      </c>
+      <c r="B2">
+        <v>0.4883638963892026</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G3043"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Rerun pipeline end to end
</commit_message>
<xml_diff>
--- a/01_Preprocess/02_Quantification/c_data/02_quantify.xlsx
+++ b/01_Preprocess/02_Quantification/c_data/02_quantify.xlsx
@@ -7,8 +7,9 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="dpc_parameters" sheetId="1" r:id="rId1"/>
-    <sheet name="protein_quality" sheetId="2" r:id="rId2"/>
+    <sheet name="overview" sheetId="1" r:id="rId1"/>
+    <sheet name="dpc_parameters" sheetId="2" r:id="rId2"/>
+    <sheet name="protein_quality" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -352,27 +353,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>intercept</t>
+          <t>sheet</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>slope</t>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>columns</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>-8.958339019700954</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dpc_parameters</t>
+        </is>
       </c>
       <c r="B2">
-        <v>0.4883638963892026</v>
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Intercept and slope of the fitted detection probability curve</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>protein_quality</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>3042</v>
+      </c>
+      <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Per protein: precursors, observed proportion, mean abundance, standard error, observations</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -382,6 +421,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>intercept</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>slope</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>-8.958339019700954</v>
+      </c>
+      <c r="B2">
+        <v>0.4883638963892026</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G3043"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>